<commit_message>
Fix /blog prerender crash from corrupted listicle dates
Re-saving the workbook dropped the number-formatting on the two
existing listicles' reviewed_date/published_date cells, so they read
back as raw Excel serials (46280) and were imported to Sanity as
"46280". formatDate() then did new Date("46280T00:00:00Z") -> Invalid
Date -> RangeError, crashing the /blog static prerender.

- Normalize those 4 cells back to ISO text (2026-09-15) in the workbook
  and re-import to Sanity.
- Harden formatDate/parseDate (BlogCollection) and longDate
  (ListicleTemplate) to accept plain dates or full ISO datetimes and
  fall back gracefully instead of throwing, so one bad CMS date can
  never fail the build again.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MaximusLabs listicle feed.xlsx
+++ b/MaximusLabs listicle feed.xlsx
@@ -6217,11 +6217,11 @@
       <c r="I2" t="str">
         <v>Published by MaximusLabs.ai, which competes with every firm listed. Listed first as publisher; signal rank fourth, printed on our own card. Read the methodology before using the order as a recommendation.</v>
       </c>
-      <c r="J2">
-        <v>46280</v>
-      </c>
-      <c r="K2">
-        <v>46280</v>
+      <c r="J2" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2026-09-15</v>
       </c>
       <c r="L2" t="str">
         <v>Not scraped from other people's rankings. Here is the actual sequence, and what was thrown away at each step.</v>
@@ -6279,11 +6279,11 @@
       <c r="I3" t="str">
         <v>Published by MaximusLabs.ai, which competes with every firm listed. Listed first as publisher; signal rank eighth, printed on our own card. Read the methodology before using the order as a recommendation.</v>
       </c>
-      <c r="J3">
-        <v>46280</v>
-      </c>
-      <c r="K3">
-        <v>46280</v>
+      <c r="J3" t="str">
+        <v>2026-09-15</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-09-15</v>
       </c>
       <c r="L3" t="str">
         <v>Built from answer engine capability first, then filtered for B2B SaaS proof. The process separates an agency's general AI-search strength from evidence that it can work in software categories and connect visibility to pipeline, signups, or recurring revenue.</v>

</xml_diff>